<commit_message>
Add Nifty hedging workflow, trades monitor, and PnL tab
</commit_message>
<xml_diff>
--- a/hols.xlsx
+++ b/hols.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rishi\projects\fit_sensex\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42C555F0-E171-445A-88F0-C9D85A596B8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA004A15-25E6-4E63-8127-F87FF4817FFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{9BA601C2-EC50-4BAB-A3C9-5F4284071222}"/>
+    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{9BA601C2-EC50-4BAB-A3C9-5F4284071222}"/>
   </bookViews>
   <sheets>
     <sheet name="hols " sheetId="2" r:id="rId1"/>
-    <sheet name="params" sheetId="1" r:id="rId2"/>
+    <sheet name="variables_sensex" sheetId="3" r:id="rId2"/>
+    <sheet name="variables_nifty" sheetId="4" r:id="rId3"/>
+    <sheet name="params_sensex" sheetId="1" r:id="rId4"/>
+    <sheet name="params_nifty" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="CET">#REF!</definedName>
@@ -43,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="72">
   <si>
     <t>Isholiday</t>
   </si>
@@ -155,6 +158,111 @@
   <si>
     <t>floorR</t>
   </si>
+  <si>
+    <t>Input</t>
+  </si>
+  <si>
+    <t>Default value</t>
+  </si>
+  <si>
+    <t>Env override</t>
+  </si>
+  <si>
+    <t>Low Strike</t>
+  </si>
+  <si>
+    <t>LOW_STRIKE</t>
+  </si>
+  <si>
+    <t>High Strike</t>
+  </si>
+  <si>
+    <t>HIGH_STRIKE</t>
+  </si>
+  <si>
+    <t>Strike Gap</t>
+  </si>
+  <si>
+    <t>STRIKE_GAP</t>
+  </si>
+  <si>
+    <t>Initial User Value</t>
+  </si>
+  <si>
+    <t>USER_VALUE</t>
+  </si>
+  <si>
+    <t>Calendar Days</t>
+  </si>
+  <si>
+    <t>CALENDAR_DAYS</t>
+  </si>
+  <si>
+    <t>Intraday Var</t>
+  </si>
+  <si>
+    <t>INTRADAY_VAR</t>
+  </si>
+  <si>
+    <t>Funding Rate</t>
+  </si>
+  <si>
+    <t>FUNDING_RATE</t>
+  </si>
+  <si>
+    <t>Brokerage Rate</t>
+  </si>
+  <si>
+    <t>BROKERAGE_RATE</t>
+  </si>
+  <si>
+    <t>Risk Free Rate</t>
+  </si>
+  <si>
+    <t>RISK_FREE_RATE</t>
+  </si>
+  <si>
+    <t>Initial ATM Vol</t>
+  </si>
+  <si>
+    <t>ATM_VOL</t>
+  </si>
+  <si>
+    <t>GUI Refresh</t>
+  </si>
+  <si>
+    <t>REFRESH_MS</t>
+  </si>
+  <si>
+    <t>Kite Exchange</t>
+  </si>
+  <si>
+    <t>BFO</t>
+  </si>
+  <si>
+    <t>KITE_EXCHANGE</t>
+  </si>
+  <si>
+    <t>Symbol Name</t>
+  </si>
+  <si>
+    <t>SENSEX</t>
+  </si>
+  <si>
+    <t>SYMBOL_NAME</t>
+  </si>
+  <si>
+    <t>1000 ms</t>
+  </si>
+  <si>
+    <t>NFO</t>
+  </si>
+  <si>
+    <t>NIFTY</t>
+  </si>
+  <si>
+    <t>Delta Hedge Threshold Ratio</t>
+  </si>
 </sst>
 </file>
 
@@ -164,7 +272,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="#,##0.00_ ;[Red]\-#,##0.00\ "/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -188,6 +296,18 @@
     <font>
       <sz val="14"/>
       <color rgb="FF44475B"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1A1C1F"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1A1C1F"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -251,7 +371,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -287,6 +407,27 @@
     </xf>
     <xf numFmtId="2" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -715,11 +856,11 @@
     <row r="3" spans="1:24" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="8">
         <f ca="1">TODAY()</f>
-        <v>46153</v>
+        <v>46155</v>
       </c>
       <c r="B3" s="4">
         <f ca="1">+VLOOKUP(A3,H:M,6,FALSE)</f>
-        <v>91.5</v>
+        <v>93.5</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>12</v>
@@ -823,7 +964,7 @@
       </c>
       <c r="C5" s="16">
         <f t="shared" ref="C5:C15" ca="1" si="8">+B5-$B$3</f>
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="D5">
         <f>VLOOKUP(A5,$H:$I,2,FALSE)</f>
@@ -881,7 +1022,7 @@
       </c>
       <c r="C6" s="16">
         <f t="shared" ca="1" si="8"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D6">
         <f t="shared" ref="D6:D15" si="9">VLOOKUP(A6,$H:$I,2,FALSE)</f>
@@ -939,7 +1080,7 @@
       </c>
       <c r="C7" s="16">
         <f t="shared" ca="1" si="8"/>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D7">
         <f t="shared" si="9"/>
@@ -997,7 +1138,7 @@
       </c>
       <c r="C8" s="16">
         <f t="shared" ca="1" si="8"/>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D8">
         <f t="shared" si="9"/>
@@ -1055,7 +1196,7 @@
       </c>
       <c r="C9" s="16">
         <f t="shared" ca="1" si="8"/>
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D9">
         <f t="shared" si="9"/>
@@ -1113,7 +1254,7 @@
       </c>
       <c r="C10" s="16">
         <f t="shared" ca="1" si="8"/>
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D10">
         <f t="shared" si="9"/>
@@ -1171,7 +1312,7 @@
       </c>
       <c r="C11" s="16">
         <f t="shared" ca="1" si="8"/>
-        <v>15.5</v>
+        <v>13.5</v>
       </c>
       <c r="D11">
         <f t="shared" si="9"/>
@@ -1229,7 +1370,7 @@
       </c>
       <c r="C12" s="16">
         <f t="shared" ca="1" si="8"/>
-        <v>17.5</v>
+        <v>15.5</v>
       </c>
       <c r="D12">
         <f t="shared" si="9"/>
@@ -1287,7 +1428,7 @@
       </c>
       <c r="C13" s="16">
         <f t="shared" ca="1" si="8"/>
-        <v>20.5</v>
+        <v>18.5</v>
       </c>
       <c r="D13">
         <f t="shared" si="9"/>
@@ -1345,7 +1486,7 @@
       </c>
       <c r="C14" s="16">
         <f t="shared" ca="1" si="8"/>
-        <v>22.5</v>
+        <v>20.5</v>
       </c>
       <c r="D14">
         <f t="shared" si="9"/>
@@ -1403,7 +1544,7 @@
       </c>
       <c r="C15" s="16">
         <f t="shared" ca="1" si="8"/>
-        <v>25.5</v>
+        <v>23.5</v>
       </c>
       <c r="D15">
         <f t="shared" si="9"/>
@@ -1461,7 +1602,7 @@
       </c>
       <c r="C16" s="16">
         <f t="shared" ref="C16:C72" ca="1" si="11">+B16-$B$3</f>
-        <v>27.5</v>
+        <v>25.5</v>
       </c>
       <c r="D16">
         <f t="shared" ref="D16:D33" si="12">VLOOKUP(A16,$H:$I,2,FALSE)</f>
@@ -1519,7 +1660,7 @@
       </c>
       <c r="C17" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>30.5</v>
+        <v>28.5</v>
       </c>
       <c r="D17">
         <f t="shared" si="12"/>
@@ -1577,7 +1718,7 @@
       </c>
       <c r="C18" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>32.5</v>
+        <v>30.5</v>
       </c>
       <c r="D18">
         <f t="shared" si="12"/>
@@ -1635,7 +1776,7 @@
       </c>
       <c r="C19" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D19">
         <f t="shared" si="12"/>
@@ -1683,7 +1824,7 @@
       </c>
       <c r="C20" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D20">
         <f t="shared" si="12"/>
@@ -1728,7 +1869,7 @@
       </c>
       <c r="C21" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D21">
         <f t="shared" si="12"/>
@@ -1773,7 +1914,7 @@
       </c>
       <c r="C22" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D22">
         <f t="shared" si="12"/>
@@ -1818,7 +1959,7 @@
       </c>
       <c r="C23" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D23">
         <f t="shared" si="12"/>
@@ -1863,7 +2004,7 @@
       </c>
       <c r="C24" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D24">
         <f t="shared" si="12"/>
@@ -1909,7 +2050,7 @@
       </c>
       <c r="C25" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D25">
         <f t="shared" si="12"/>
@@ -1954,7 +2095,7 @@
       </c>
       <c r="C26" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D26">
         <f t="shared" si="12"/>
@@ -1999,7 +2140,7 @@
       </c>
       <c r="C27" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D27">
         <f t="shared" si="12"/>
@@ -2044,7 +2185,7 @@
       </c>
       <c r="C28" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D28">
         <f t="shared" si="12"/>
@@ -2091,7 +2232,7 @@
       </c>
       <c r="C29" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D29">
         <f t="shared" si="12"/>
@@ -2137,7 +2278,7 @@
       </c>
       <c r="C30" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D30">
         <f t="shared" si="12"/>
@@ -2183,7 +2324,7 @@
       </c>
       <c r="C31" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D31">
         <f t="shared" si="12"/>
@@ -2229,7 +2370,7 @@
       </c>
       <c r="C32" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D32">
         <f t="shared" si="12"/>
@@ -2274,7 +2415,7 @@
       </c>
       <c r="C33" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D33">
         <f t="shared" si="12"/>
@@ -2319,7 +2460,7 @@
       </c>
       <c r="C34" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D34">
         <f t="shared" ref="D34:D72" si="14">VLOOKUP(A34,$H:$I,2,FALSE)</f>
@@ -2364,7 +2505,7 @@
       </c>
       <c r="C35" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D35">
         <f t="shared" si="14"/>
@@ -2409,7 +2550,7 @@
       </c>
       <c r="C36" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D36">
         <f t="shared" si="14"/>
@@ -2455,7 +2596,7 @@
       </c>
       <c r="C37" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D37">
         <f t="shared" si="14"/>
@@ -2501,7 +2642,7 @@
       </c>
       <c r="C38" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D38">
         <f t="shared" si="14"/>
@@ -2547,7 +2688,7 @@
       </c>
       <c r="C39" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D39">
         <f t="shared" si="14"/>
@@ -2593,7 +2734,7 @@
       </c>
       <c r="C40" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D40">
         <f t="shared" si="14"/>
@@ -2639,7 +2780,7 @@
       </c>
       <c r="C41" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>89.5</v>
+        <v>87.5</v>
       </c>
       <c r="D41">
         <f t="shared" si="14"/>
@@ -2685,7 +2826,7 @@
       </c>
       <c r="C42" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>91.5</v>
+        <v>89.5</v>
       </c>
       <c r="D42">
         <f t="shared" si="14"/>
@@ -2731,7 +2872,7 @@
       </c>
       <c r="C43" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>94.5</v>
+        <v>92.5</v>
       </c>
       <c r="D43">
         <f t="shared" si="14"/>
@@ -2777,7 +2918,7 @@
       </c>
       <c r="C44" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>96.5</v>
+        <v>94.5</v>
       </c>
       <c r="D44">
         <f t="shared" si="14"/>
@@ -2823,7 +2964,7 @@
       </c>
       <c r="C45" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>99.5</v>
+        <v>97.5</v>
       </c>
       <c r="D45">
         <f t="shared" si="14"/>
@@ -2869,7 +3010,7 @@
       </c>
       <c r="C46" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>101.5</v>
+        <v>99.5</v>
       </c>
       <c r="D46">
         <f t="shared" si="14"/>
@@ -2915,7 +3056,7 @@
       </c>
       <c r="C47" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D47">
         <f t="shared" si="14"/>
@@ -2961,7 +3102,7 @@
       </c>
       <c r="C48" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D48">
         <f t="shared" si="14"/>
@@ -3006,7 +3147,7 @@
       </c>
       <c r="C49" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D49">
         <f t="shared" si="14"/>
@@ -3051,7 +3192,7 @@
       </c>
       <c r="C50" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D50">
         <f t="shared" si="14"/>
@@ -3096,7 +3237,7 @@
       </c>
       <c r="C51" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D51">
         <f t="shared" si="14"/>
@@ -3141,7 +3282,7 @@
       </c>
       <c r="C52" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>115.5</v>
+        <v>113.5</v>
       </c>
       <c r="D52">
         <f t="shared" si="14"/>
@@ -3186,7 +3327,7 @@
       </c>
       <c r="C53" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>118.5</v>
+        <v>116.5</v>
       </c>
       <c r="D53">
         <f t="shared" si="14"/>
@@ -3231,7 +3372,7 @@
       </c>
       <c r="C54" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>120.5</v>
+        <v>118.5</v>
       </c>
       <c r="D54">
         <f t="shared" si="14"/>
@@ -3276,7 +3417,7 @@
       </c>
       <c r="C55" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>123.5</v>
+        <v>121.5</v>
       </c>
       <c r="D55">
         <f t="shared" si="14"/>
@@ -3321,7 +3462,7 @@
       </c>
       <c r="C56" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>125.5</v>
+        <v>123.5</v>
       </c>
       <c r="D56">
         <f t="shared" si="14"/>
@@ -3366,7 +3507,7 @@
       </c>
       <c r="C57" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>127.5</v>
+        <v>125.5</v>
       </c>
       <c r="D57">
         <f t="shared" si="14"/>
@@ -3411,7 +3552,7 @@
       </c>
       <c r="C58" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D58">
         <f t="shared" si="14"/>
@@ -3456,7 +3597,7 @@
       </c>
       <c r="C59" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D59">
         <f t="shared" si="14"/>
@@ -3501,7 +3642,7 @@
       </c>
       <c r="C60" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D60">
         <f t="shared" si="14"/>
@@ -3546,7 +3687,7 @@
       </c>
       <c r="C61" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D61">
         <f t="shared" si="14"/>
@@ -3591,7 +3732,7 @@
       </c>
       <c r="C62" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>139.5</v>
+        <v>137.5</v>
       </c>
       <c r="D62">
         <f t="shared" si="14"/>
@@ -3636,7 +3777,7 @@
       </c>
       <c r="C63" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>142.5</v>
+        <v>140.5</v>
       </c>
       <c r="D63">
         <f t="shared" si="14"/>
@@ -3681,7 +3822,7 @@
       </c>
       <c r="C64" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>144.5</v>
+        <v>142.5</v>
       </c>
       <c r="D64">
         <f t="shared" si="14"/>
@@ -3726,7 +3867,7 @@
       </c>
       <c r="C65" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>147.5</v>
+        <v>145.5</v>
       </c>
       <c r="D65">
         <f t="shared" si="14"/>
@@ -3771,7 +3912,7 @@
       </c>
       <c r="C66" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>149.5</v>
+        <v>147.5</v>
       </c>
       <c r="D66">
         <f t="shared" si="14"/>
@@ -3816,7 +3957,7 @@
       </c>
       <c r="C67" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>152.5</v>
+        <v>150.5</v>
       </c>
       <c r="D67">
         <f t="shared" si="14"/>
@@ -3861,7 +4002,7 @@
       </c>
       <c r="C68" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>154.5</v>
+        <v>152.5</v>
       </c>
       <c r="D68">
         <f t="shared" si="14"/>
@@ -3906,7 +4047,7 @@
       </c>
       <c r="C69" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>157.5</v>
+        <v>155.5</v>
       </c>
       <c r="D69">
         <f t="shared" si="14"/>
@@ -3951,7 +4092,7 @@
       </c>
       <c r="C70" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>159.5</v>
+        <v>157.5</v>
       </c>
       <c r="D70">
         <f t="shared" si="14"/>
@@ -3996,7 +4137,7 @@
       </c>
       <c r="C71" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D71">
         <f t="shared" si="14"/>
@@ -4041,7 +4182,7 @@
       </c>
       <c r="C72" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="D72">
         <f t="shared" si="14"/>
@@ -13376,6 +13517,374 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0685B118-9C79-451E-8585-AEC419BB466D}">
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.140625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="18.28515625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="24.140625" style="21" customWidth="1"/>
+    <col min="4" max="16384" width="9.140625" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" s="20" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="22">
+        <v>65000</v>
+      </c>
+      <c r="C2" s="23" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="B3" s="22">
+        <v>85000</v>
+      </c>
+      <c r="C3" s="23" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" s="22">
+        <v>100</v>
+      </c>
+      <c r="C4" s="23" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5" s="22">
+        <v>76300</v>
+      </c>
+      <c r="C5" s="23" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="B6" s="22">
+        <v>255.5</v>
+      </c>
+      <c r="C6" s="23" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="B7" s="22">
+        <v>0.4</v>
+      </c>
+      <c r="C7" s="23" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="B8" s="22">
+        <v>5.5E-2</v>
+      </c>
+      <c r="C8" s="23" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" s="22">
+        <v>0</v>
+      </c>
+      <c r="C9" s="23" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="B10" s="22">
+        <v>5.5E-2</v>
+      </c>
+      <c r="C10" s="23" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="B11" s="22">
+        <v>0.17599999999999999</v>
+      </c>
+      <c r="C11" s="23" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="B12" s="22" t="s">
+        <v>68</v>
+      </c>
+      <c r="C12" s="23" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="B13" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C13" s="23" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="B14" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="C14" s="23" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="B15" s="22">
+        <v>0.5</v>
+      </c>
+      <c r="C15" s="23"/>
+    </row>
+    <row r="16" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="18"/>
+      <c r="B16" s="22"/>
+      <c r="C16" s="23"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB543FF4-ECA7-4AC0-ABF4-7EB91A23751E}">
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="27.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.28515625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="24.140625" style="21" customWidth="1"/>
+    <col min="4" max="16384" width="9.140625" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" s="20" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="22">
+        <v>21000</v>
+      </c>
+      <c r="C2" s="23" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="B3" s="22">
+        <v>26500</v>
+      </c>
+      <c r="C3" s="23" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" s="22">
+        <v>50</v>
+      </c>
+      <c r="C4" s="23" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5" s="22">
+        <v>23500</v>
+      </c>
+      <c r="C5" s="23" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="B6" s="22">
+        <v>255.5</v>
+      </c>
+      <c r="C6" s="23" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="B7" s="22">
+        <v>0.4</v>
+      </c>
+      <c r="C7" s="23" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="B8" s="22">
+        <v>5.5E-2</v>
+      </c>
+      <c r="C8" s="23" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" s="22">
+        <v>0</v>
+      </c>
+      <c r="C9" s="23" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="B10" s="22">
+        <v>5.5E-2</v>
+      </c>
+      <c r="C10" s="23" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="B11" s="22">
+        <v>0.17599999999999999</v>
+      </c>
+      <c r="C11" s="23" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="B12" s="22" t="s">
+        <v>68</v>
+      </c>
+      <c r="C12" s="23" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="B13" s="19" t="s">
+        <v>69</v>
+      </c>
+      <c r="C13" s="23" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="B14" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="C14" s="23" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="B15" s="22">
+        <v>0.5</v>
+      </c>
+      <c r="C15" s="23"/>
+    </row>
+    <row r="16" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="18"/>
+      <c r="B16" s="22"/>
+      <c r="C16" s="23"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04D2A993-3FF5-48EE-98A7-DB4BC5B4CDE7}">
   <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -13385,6 +13894,56 @@
         <v>32</v>
       </c>
       <c r="B1">
+        <v>2.5000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2">
+        <v>-0.4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B3">
+        <v>-0.15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4">
+        <v>0.41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5">
+        <v>-0.53</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2009890E-8F2C-425B-BDB9-A1D61B2D2E26}">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1">
         <v>4.4999999999999998E-2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update hedge threshold controls and PnL workflow
</commit_message>
<xml_diff>
--- a/hols.xlsx
+++ b/hols.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rishi\projects\fit_sensex\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA004A15-25E6-4E63-8127-F87FF4817FFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EDC1290-6716-4DE2-A2D3-00A13EA7BB64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{9BA601C2-EC50-4BAB-A3C9-5F4284071222}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9BA601C2-EC50-4BAB-A3C9-5F4284071222}"/>
   </bookViews>
   <sheets>
     <sheet name="hols " sheetId="2" r:id="rId1"/>
@@ -856,11 +856,11 @@
     <row r="3" spans="1:24" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="8">
         <f ca="1">TODAY()</f>
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B3" s="4">
         <f ca="1">+VLOOKUP(A3,H:M,6,FALSE)</f>
-        <v>93.5</v>
+        <v>94.5</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>12</v>
@@ -964,7 +964,7 @@
       </c>
       <c r="C5" s="16">
         <f t="shared" ref="C5:C15" ca="1" si="8">+B5-$B$3</f>
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="D5">
         <f>VLOOKUP(A5,$H:$I,2,FALSE)</f>
@@ -1022,7 +1022,7 @@
       </c>
       <c r="C6" s="16">
         <f t="shared" ca="1" si="8"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6">
         <f t="shared" ref="D6:D15" si="9">VLOOKUP(A6,$H:$I,2,FALSE)</f>
@@ -1080,7 +1080,7 @@
       </c>
       <c r="C7" s="16">
         <f t="shared" ca="1" si="8"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D7">
         <f t="shared" si="9"/>
@@ -1138,7 +1138,7 @@
       </c>
       <c r="C8" s="16">
         <f t="shared" ca="1" si="8"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D8">
         <f t="shared" si="9"/>
@@ -1196,7 +1196,7 @@
       </c>
       <c r="C9" s="16">
         <f t="shared" ca="1" si="8"/>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D9">
         <f t="shared" si="9"/>
@@ -1254,7 +1254,7 @@
       </c>
       <c r="C10" s="16">
         <f t="shared" ca="1" si="8"/>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D10">
         <f t="shared" si="9"/>
@@ -1312,7 +1312,7 @@
       </c>
       <c r="C11" s="16">
         <f t="shared" ca="1" si="8"/>
-        <v>13.5</v>
+        <v>12.5</v>
       </c>
       <c r="D11">
         <f t="shared" si="9"/>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="C12" s="16">
         <f t="shared" ca="1" si="8"/>
-        <v>15.5</v>
+        <v>14.5</v>
       </c>
       <c r="D12">
         <f t="shared" si="9"/>
@@ -1428,7 +1428,7 @@
       </c>
       <c r="C13" s="16">
         <f t="shared" ca="1" si="8"/>
-        <v>18.5</v>
+        <v>17.5</v>
       </c>
       <c r="D13">
         <f t="shared" si="9"/>
@@ -1486,7 +1486,7 @@
       </c>
       <c r="C14" s="16">
         <f t="shared" ca="1" si="8"/>
-        <v>20.5</v>
+        <v>19.5</v>
       </c>
       <c r="D14">
         <f t="shared" si="9"/>
@@ -1544,7 +1544,7 @@
       </c>
       <c r="C15" s="16">
         <f t="shared" ca="1" si="8"/>
-        <v>23.5</v>
+        <v>22.5</v>
       </c>
       <c r="D15">
         <f t="shared" si="9"/>
@@ -1602,7 +1602,7 @@
       </c>
       <c r="C16" s="16">
         <f t="shared" ref="C16:C72" ca="1" si="11">+B16-$B$3</f>
-        <v>25.5</v>
+        <v>24.5</v>
       </c>
       <c r="D16">
         <f t="shared" ref="D16:D33" si="12">VLOOKUP(A16,$H:$I,2,FALSE)</f>
@@ -1660,7 +1660,7 @@
       </c>
       <c r="C17" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>28.5</v>
+        <v>27.5</v>
       </c>
       <c r="D17">
         <f t="shared" si="12"/>
@@ -1718,7 +1718,7 @@
       </c>
       <c r="C18" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>30.5</v>
+        <v>29.5</v>
       </c>
       <c r="D18">
         <f t="shared" si="12"/>
@@ -1776,7 +1776,7 @@
       </c>
       <c r="C19" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D19">
         <f t="shared" si="12"/>
@@ -1824,7 +1824,7 @@
       </c>
       <c r="C20" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D20">
         <f t="shared" si="12"/>
@@ -1869,7 +1869,7 @@
       </c>
       <c r="C21" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D21">
         <f t="shared" si="12"/>
@@ -1914,7 +1914,7 @@
       </c>
       <c r="C22" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D22">
         <f t="shared" si="12"/>
@@ -1959,7 +1959,7 @@
       </c>
       <c r="C23" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D23">
         <f t="shared" si="12"/>
@@ -2004,7 +2004,7 @@
       </c>
       <c r="C24" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D24">
         <f t="shared" si="12"/>
@@ -2050,7 +2050,7 @@
       </c>
       <c r="C25" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D25">
         <f t="shared" si="12"/>
@@ -2095,7 +2095,7 @@
       </c>
       <c r="C26" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D26">
         <f t="shared" si="12"/>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="C27" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D27">
         <f t="shared" si="12"/>
@@ -2185,7 +2185,7 @@
       </c>
       <c r="C28" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D28">
         <f t="shared" si="12"/>
@@ -2232,7 +2232,7 @@
       </c>
       <c r="C29" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D29">
         <f t="shared" si="12"/>
@@ -2278,7 +2278,7 @@
       </c>
       <c r="C30" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D30">
         <f t="shared" si="12"/>
@@ -2324,7 +2324,7 @@
       </c>
       <c r="C31" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D31">
         <f t="shared" si="12"/>
@@ -2370,7 +2370,7 @@
       </c>
       <c r="C32" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D32">
         <f t="shared" si="12"/>
@@ -2415,7 +2415,7 @@
       </c>
       <c r="C33" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D33">
         <f t="shared" si="12"/>
@@ -2460,7 +2460,7 @@
       </c>
       <c r="C34" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D34">
         <f t="shared" ref="D34:D72" si="14">VLOOKUP(A34,$H:$I,2,FALSE)</f>
@@ -2505,7 +2505,7 @@
       </c>
       <c r="C35" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D35">
         <f t="shared" si="14"/>
@@ -2550,7 +2550,7 @@
       </c>
       <c r="C36" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D36">
         <f t="shared" si="14"/>
@@ -2596,7 +2596,7 @@
       </c>
       <c r="C37" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D37">
         <f t="shared" si="14"/>
@@ -2642,7 +2642,7 @@
       </c>
       <c r="C38" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D38">
         <f t="shared" si="14"/>
@@ -2688,7 +2688,7 @@
       </c>
       <c r="C39" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D39">
         <f t="shared" si="14"/>
@@ -2734,7 +2734,7 @@
       </c>
       <c r="C40" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D40">
         <f t="shared" si="14"/>
@@ -2780,7 +2780,7 @@
       </c>
       <c r="C41" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>87.5</v>
+        <v>86.5</v>
       </c>
       <c r="D41">
         <f t="shared" si="14"/>
@@ -2826,7 +2826,7 @@
       </c>
       <c r="C42" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>89.5</v>
+        <v>88.5</v>
       </c>
       <c r="D42">
         <f t="shared" si="14"/>
@@ -2872,7 +2872,7 @@
       </c>
       <c r="C43" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>92.5</v>
+        <v>91.5</v>
       </c>
       <c r="D43">
         <f t="shared" si="14"/>
@@ -2918,7 +2918,7 @@
       </c>
       <c r="C44" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>94.5</v>
+        <v>93.5</v>
       </c>
       <c r="D44">
         <f t="shared" si="14"/>
@@ -2964,7 +2964,7 @@
       </c>
       <c r="C45" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>97.5</v>
+        <v>96.5</v>
       </c>
       <c r="D45">
         <f t="shared" si="14"/>
@@ -3010,7 +3010,7 @@
       </c>
       <c r="C46" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>99.5</v>
+        <v>98.5</v>
       </c>
       <c r="D46">
         <f t="shared" si="14"/>
@@ -3056,7 +3056,7 @@
       </c>
       <c r="C47" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D47">
         <f t="shared" si="14"/>
@@ -3102,7 +3102,7 @@
       </c>
       <c r="C48" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D48">
         <f t="shared" si="14"/>
@@ -3147,7 +3147,7 @@
       </c>
       <c r="C49" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D49">
         <f t="shared" si="14"/>
@@ -3192,7 +3192,7 @@
       </c>
       <c r="C50" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D50">
         <f t="shared" si="14"/>
@@ -3237,7 +3237,7 @@
       </c>
       <c r="C51" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D51">
         <f t="shared" si="14"/>
@@ -3282,7 +3282,7 @@
       </c>
       <c r="C52" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>113.5</v>
+        <v>112.5</v>
       </c>
       <c r="D52">
         <f t="shared" si="14"/>
@@ -3327,7 +3327,7 @@
       </c>
       <c r="C53" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>116.5</v>
+        <v>115.5</v>
       </c>
       <c r="D53">
         <f t="shared" si="14"/>
@@ -3372,7 +3372,7 @@
       </c>
       <c r="C54" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>118.5</v>
+        <v>117.5</v>
       </c>
       <c r="D54">
         <f t="shared" si="14"/>
@@ -3417,7 +3417,7 @@
       </c>
       <c r="C55" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>121.5</v>
+        <v>120.5</v>
       </c>
       <c r="D55">
         <f t="shared" si="14"/>
@@ -3462,7 +3462,7 @@
       </c>
       <c r="C56" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>123.5</v>
+        <v>122.5</v>
       </c>
       <c r="D56">
         <f t="shared" si="14"/>
@@ -3507,7 +3507,7 @@
       </c>
       <c r="C57" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>125.5</v>
+        <v>124.5</v>
       </c>
       <c r="D57">
         <f t="shared" si="14"/>
@@ -3552,7 +3552,7 @@
       </c>
       <c r="C58" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D58">
         <f t="shared" si="14"/>
@@ -3597,7 +3597,7 @@
       </c>
       <c r="C59" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D59">
         <f t="shared" si="14"/>
@@ -3642,7 +3642,7 @@
       </c>
       <c r="C60" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D60">
         <f t="shared" si="14"/>
@@ -3687,7 +3687,7 @@
       </c>
       <c r="C61" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D61">
         <f t="shared" si="14"/>
@@ -3732,7 +3732,7 @@
       </c>
       <c r="C62" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>137.5</v>
+        <v>136.5</v>
       </c>
       <c r="D62">
         <f t="shared" si="14"/>
@@ -3777,7 +3777,7 @@
       </c>
       <c r="C63" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>140.5</v>
+        <v>139.5</v>
       </c>
       <c r="D63">
         <f t="shared" si="14"/>
@@ -3822,7 +3822,7 @@
       </c>
       <c r="C64" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>142.5</v>
+        <v>141.5</v>
       </c>
       <c r="D64">
         <f t="shared" si="14"/>
@@ -3867,7 +3867,7 @@
       </c>
       <c r="C65" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>145.5</v>
+        <v>144.5</v>
       </c>
       <c r="D65">
         <f t="shared" si="14"/>
@@ -3912,7 +3912,7 @@
       </c>
       <c r="C66" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>147.5</v>
+        <v>146.5</v>
       </c>
       <c r="D66">
         <f t="shared" si="14"/>
@@ -3957,7 +3957,7 @@
       </c>
       <c r="C67" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>150.5</v>
+        <v>149.5</v>
       </c>
       <c r="D67">
         <f t="shared" si="14"/>
@@ -4002,7 +4002,7 @@
       </c>
       <c r="C68" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>152.5</v>
+        <v>151.5</v>
       </c>
       <c r="D68">
         <f t="shared" si="14"/>
@@ -4047,7 +4047,7 @@
       </c>
       <c r="C69" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>155.5</v>
+        <v>154.5</v>
       </c>
       <c r="D69">
         <f t="shared" si="14"/>
@@ -4092,7 +4092,7 @@
       </c>
       <c r="C70" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>157.5</v>
+        <v>156.5</v>
       </c>
       <c r="D70">
         <f t="shared" si="14"/>
@@ -4137,7 +4137,7 @@
       </c>
       <c r="C71" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D71">
         <f t="shared" si="14"/>
@@ -4182,7 +4182,7 @@
       </c>
       <c r="C72" s="16">
         <f t="shared" ca="1" si="11"/>
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D72">
         <f t="shared" si="14"/>

</xml_diff>